<commit_message>
[session] read simplified esklp headers
</commit_message>
<xml_diff>
--- a/data/esklp_test/esklp_smnn_test.xlsx
+++ b/data/esklp_test/esklp_smnn_test.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="esklp_smnn_test" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,276 +413,378 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>meta 1</t>
+          <t>Стандартизованное МНН</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Код узла СМНН</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Стандартизованная лекарственная форма</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Стандартизованная дозировка кол-во</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Единица измерения</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Наименование единицы из ОКЕИ</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Единица измерения лекарственного препарата</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Наименование ФТГ</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>код АТХ</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ЖНВЛП</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Список нормализованных МНН для узла СМНН</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Список нормализованных лекарственных форм и дозировок для узла СМНН</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>meta 2</t>
+          <t>Ибупрофен</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SMNN-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>таблетки</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>миллиграмм</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Нестероидные противовоспалительные препараты</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>M01AE</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Ибупрофен</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Ибупрофен</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>таблетки 200 мг</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>meta 3</t>
+          <t>Парацетамол</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SMNN-002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>таблетки</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>миллиграмм</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Анальгезирующее ненаркотическое средство</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>N02BE01</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Парацетамол</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Парацетамол</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>таблетки 500 мг</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>meta 4</t>
+          <t>Колекальциферол</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SMNN-003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>капли для приема внутрь</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>МЕ/мл</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>МЕ/мл</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Кальциево-фосфорного обмена регулятор</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>A11CC05</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Колекальциферол</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Колекальциферол</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>капли 15000 МЕ/мл</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>col1</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>col2</t>
+          <t>SMNN-004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>col3</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>col4</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>col5</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>col6</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>col7</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>col8</t>
-        </is>
-      </c>
+          <t>пластырь</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>col9</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>col10</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>col11</t>
-        </is>
-      </c>
+          <t>Медицинские изделия</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>col12</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>col13</t>
-        </is>
-      </c>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>col14</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>col15</t>
+          <t>пластырь</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Гиалуроновая кислота</t>
+        </is>
+      </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SMNN001</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+          <t>SMNN-005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>раствор для внутрисуставного введения</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>мг/мл</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>мг/мл</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Средства для лечения заболеваний опорно-двигательного аппарата</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>M09AX</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Гиалуроновая кислота</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Нестероидные противовоспалительные препараты</t>
+          <t>Гиалуроновая кислота</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>M01AE</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Производные пропионовой кислоты</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>SMNN002</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>анальгезирующее ненаркотическое средство</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>N02BE</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Анилиды</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>SMNN003</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>анальгезирующее комбинированное средство</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>N02BA</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Салициловая кислота и ее производные</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>SMNN004</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>антигистаминное средство системного действия</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>R06AX</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Другие антигистаминные препараты системного действия</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>SMNN005</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>антибактериальное средство пенициллинового ряда</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>J01CA</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Пенициллины с расширенным спектром действия</t>
+          <t>раствор 10 мг/мл</t>
         </is>
       </c>
     </row>

</xml_diff>